<commit_message>
chore: update environment configurations, requirements, and documentation
</commit_message>
<xml_diff>
--- a/docs/Halcyon_Credit_Daily_Dashboard.xlsx
+++ b/docs/Halcyon_Credit_Daily_Dashboard.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yash/CapStone/credit-arbiter/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{233D63A6-909C-1047-BFFA-44E7A76DC6D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72F9204B-713E-E746-935F-17C0274C8EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="253">
   <si>
     <t>Halcyon Credit — Daily Progress Dashboard</t>
   </si>
@@ -47,7 +47,7 @@
     <t>Agentic Underwriting Copilot  ·  Sprint 0 → Sprint 4  ·  Owner: Yash Gupta</t>
   </si>
   <si>
-    <t>Last updated: 2026-06-22</t>
+    <t>Last updated: 2026-07-07</t>
   </si>
   <si>
     <t>KEY METRICS</t>
@@ -65,42 +65,45 @@
     <t>Stories Done</t>
   </si>
   <si>
+    <t>Sprint 2</t>
+  </si>
+  <si>
+    <t>Open Blockers</t>
+  </si>
+  <si>
+    <t>Pending Tasks</t>
+  </si>
+  <si>
+    <t>High Priority Items</t>
+  </si>
+  <si>
+    <t>Days into Project</t>
+  </si>
+  <si>
+    <t>SPRINT PROGRESS</t>
+  </si>
+  <si>
+    <t>Sprint</t>
+  </si>
+  <si>
+    <t>Goal</t>
+  </si>
+  <si>
+    <t>Planned pts</t>
+  </si>
+  <si>
+    <t>Done pts</t>
+  </si>
+  <si>
+    <t>% Complete</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
     <t>Sprint 0</t>
   </si>
   <si>
-    <t>Open Blockers</t>
-  </si>
-  <si>
-    <t>Pending Tasks</t>
-  </si>
-  <si>
-    <t>High Priority Items</t>
-  </si>
-  <si>
-    <t>Days into Project</t>
-  </si>
-  <si>
-    <t>SPRINT PROGRESS</t>
-  </si>
-  <si>
-    <t>Sprint</t>
-  </si>
-  <si>
-    <t>Goal</t>
-  </si>
-  <si>
-    <t>Planned pts</t>
-  </si>
-  <si>
-    <t>Done pts</t>
-  </si>
-  <si>
-    <t>% Complete</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
     <t>Discovery, planning, de-risking</t>
   </si>
   <si>
@@ -110,9 +113,6 @@
     <t>POC — end-to-end thin slice</t>
   </si>
   <si>
-    <t>Sprint 2</t>
-  </si>
-  <si>
     <t>Multi-scheme policy + ML hardening</t>
   </si>
   <si>
@@ -173,10 +173,25 @@
     <t>A-8b signoff; vector store choice; wireframes</t>
   </si>
   <si>
+    <t>Yash, Abe, Het</t>
+  </si>
+  <si>
+    <t>Sprint 0 baseline pushed to repo</t>
+  </si>
+  <si>
+    <t>100%</t>
+  </si>
+  <si>
+    <t>Completed all remaining Sprint 1 stories (US-102-US-111): CSV ingestion + INCOMPLETE handling, placeholder risk scorer (A-8b compliant), 5-clause policy corpus, TF-IDF RAG retrieval (US-111 spike &gt;=85% accuracy), mock regulatory stub, recommendation engine with kill-switch, decision_record audit persistence, underwriter queue/detail/assess UI, demo script. Sprint 1 now 100% complete (39/39 pts, 11/11 stories).</t>
+  </si>
+  <si>
+    <t>None raised — real HC2018 dataset and LLM provider selection intentionally deferred to Sprint 2 (documented in claude.md)</t>
+  </si>
+  <si>
     <t>Yash</t>
   </si>
   <si>
-    <t>Sprint 0 baseline pushed to repo</t>
+    <t>Fixed 2 pre-existing env bugs (SQLAlchemy/Python 3.13, bcrypt/passlib pin). 36 tests passing. POC demoed end-to-end (queue -&gt; assess -&gt; decision -&gt; audit) in browser.</t>
   </si>
   <si>
     <t>Blocker ID</t>
@@ -206,216 +221,201 @@
     <t>High</t>
   </si>
   <si>
+    <t>Abe, Yash, Het</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>15-min call with Tech Lead to decide before Sprint 1</t>
+  </si>
+  <si>
+    <t>Task ID</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Epic</t>
+  </si>
+  <si>
+    <t>Due Date</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>US-006</t>
+  </si>
+  <si>
+    <t>End-to-End User Flow Definition</t>
+  </si>
+  <si>
+    <t>EPIC-12</t>
+  </si>
+  <si>
+    <t>Het</t>
+  </si>
+  <si>
+    <t>Paper sketch done; needs digitisation</t>
+  </si>
+  <si>
+    <t>US-007</t>
+  </si>
+  <si>
+    <t>Wireframes / Mockups</t>
+  </si>
+  <si>
+    <t>Not Started</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>US-008</t>
+  </si>
+  <si>
+    <t>EPIC-15</t>
+  </si>
+  <si>
+    <t>US-009</t>
+  </si>
+  <si>
+    <t>US-010</t>
+  </si>
+  <si>
+    <t>DB Design Planning</t>
+  </si>
+  <si>
+    <t>EPIC-10</t>
+  </si>
+  <si>
+    <t>Abe, Yash</t>
+  </si>
+  <si>
+    <t>US-011</t>
+  </si>
+  <si>
+    <t>API Contract (OpenAPI)</t>
+  </si>
+  <si>
+    <t>Depends on US-009</t>
+  </si>
+  <si>
+    <t>US-003</t>
+  </si>
+  <si>
+    <t>Stakeholder Discussions</t>
+  </si>
+  <si>
+    <t>Interviews to schedule</t>
+  </si>
+  <si>
+    <t>US-004</t>
+  </si>
+  <si>
+    <t>PRD Review &amp; Validation</t>
+  </si>
+  <si>
+    <t>Formal signoff record pending</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Why it matters</t>
+  </si>
+  <si>
+    <t>Next Action</t>
+  </si>
+  <si>
+    <t>Vector store choice (Chroma vs Pinecone)</t>
+  </si>
+  <si>
+    <t>Decision</t>
+  </si>
+  <si>
+    <t>Tech Lead</t>
+  </si>
+  <si>
     <t>Open</t>
   </si>
   <si>
-    <t>Vector store choice (Chroma vs Pinecone) blocking HL architecture + DB schema</t>
-  </si>
-  <si>
-    <t>Built back-of-envelope cost model for both at 200 apps/hr — Chroma ~30% cheaper, needs self-hosting</t>
-  </si>
-  <si>
-    <t>In Progress</t>
-  </si>
-  <si>
-    <t>15-min call with Tech Lead to decide before Sprint 1</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>Task ID</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
-    <t>Epic</t>
-  </si>
-  <si>
-    <t>Due Date</t>
-  </si>
-  <si>
-    <t>Priority</t>
-  </si>
-  <si>
-    <t>US-006</t>
-  </si>
-  <si>
-    <t>End-to-End User Flow Definition</t>
-  </si>
-  <si>
-    <t>EPIC-12</t>
-  </si>
-  <si>
-    <t>Paper sketch done; needs digitisation</t>
-  </si>
-  <si>
-    <t>US-007</t>
-  </si>
-  <si>
-    <t>Wireframes / Mockups</t>
-  </si>
-  <si>
-    <t>Not Started</t>
-  </si>
-  <si>
-    <t>US-008</t>
-  </si>
-  <si>
-    <t>Technical Feasibility Analysis</t>
-  </si>
-  <si>
-    <t>EPIC-15</t>
-  </si>
-  <si>
-    <t>Cost model started, latency budget pending</t>
-  </si>
-  <si>
-    <t>US-009</t>
-  </si>
-  <si>
-    <t>High-Level Architecture</t>
-  </si>
-  <si>
-    <t>Blocked by BL-002</t>
-  </si>
-  <si>
-    <t>US-010</t>
-  </si>
-  <si>
-    <t>DB Design Planning</t>
-  </si>
-  <si>
-    <t>EPIC-10</t>
-  </si>
-  <si>
-    <t>Awaiting vector store decision</t>
-  </si>
-  <si>
-    <t>US-011</t>
-  </si>
-  <si>
-    <t>API Contract (OpenAPI)</t>
-  </si>
-  <si>
-    <t>Depends on US-009</t>
+    <t>Drives architecture, DB schema, cost model</t>
+  </si>
+  <si>
+    <t>Reassign UX bandwidth for wireframes</t>
+  </si>
+  <si>
+    <t>Resource</t>
+  </si>
+  <si>
+    <t>PM</t>
+  </si>
+  <si>
+    <t>Sprint 0 cannot close without 4 wireframes</t>
+  </si>
+  <si>
+    <t>RAG retrieval accuracy spike plan</t>
+  </si>
+  <si>
+    <t>Risk</t>
+  </si>
+  <si>
+    <t>DS</t>
+  </si>
+  <si>
+    <t>★ riskiest PRD assumption (Risk R-1)</t>
+  </si>
+  <si>
+    <t>Draft 30-scenario eval set</t>
+  </si>
+  <si>
+    <t># Stories</t>
+  </si>
+  <si>
+    <t># Done</t>
+  </si>
+  <si>
+    <t>Start</t>
+  </si>
+  <si>
+    <t>End</t>
+  </si>
+  <si>
+    <t>Product Backlog — 54 user stories (reference, edit Status / Owner / % freely)</t>
+  </si>
+  <si>
+    <t>Story</t>
+  </si>
+  <si>
+    <t>Pts</t>
+  </si>
+  <si>
+    <t>US-001</t>
+  </si>
+  <si>
+    <t>Functional Requirement Gathering</t>
+  </si>
+  <si>
+    <t>US-002</t>
+  </si>
+  <si>
+    <t>Business Requirement Analysis</t>
   </si>
   <si>
     <t>US-005</t>
   </si>
   <si>
-    <t>US-003</t>
-  </si>
-  <si>
-    <t>Stakeholder Discussions</t>
-  </si>
-  <si>
-    <t>Interviews to schedule</t>
-  </si>
-  <si>
-    <t>US-004</t>
-  </si>
-  <si>
-    <t>PRD Review &amp; Validation</t>
-  </si>
-  <si>
-    <t>Formal signoff record pending</t>
-  </si>
-  <si>
-    <t>Item</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Why it matters</t>
-  </si>
-  <si>
-    <t>Next Action</t>
-  </si>
-  <si>
-    <t>Decision</t>
-  </si>
-  <si>
-    <t>Vector store choice (Chroma vs Pinecone)</t>
-  </si>
-  <si>
-    <t>Tech Lead</t>
-  </si>
-  <si>
-    <t>Drives architecture, DB schema, cost model</t>
-  </si>
-  <si>
-    <t>15-min call with Tech Lead</t>
-  </si>
-  <si>
-    <t>Reassign UX bandwidth for wireframes</t>
-  </si>
-  <si>
-    <t>Resource</t>
-  </si>
-  <si>
-    <t>PM</t>
-  </si>
-  <si>
-    <t>Sprint 0 cannot close without 4 wireframes</t>
-  </si>
-  <si>
-    <t>Discuss with PM in standup</t>
-  </si>
-  <si>
-    <t>RAG retrieval accuracy spike plan</t>
-  </si>
-  <si>
-    <t>Risk</t>
-  </si>
-  <si>
-    <t>DS</t>
-  </si>
-  <si>
-    <t>★ riskiest PRD assumption (Risk R-1)</t>
-  </si>
-  <si>
-    <t>Draft 30-scenario eval set</t>
-  </si>
-  <si>
-    <t># Stories</t>
-  </si>
-  <si>
-    <t># Done</t>
-  </si>
-  <si>
-    <t>Start</t>
-  </si>
-  <si>
-    <t>End</t>
-  </si>
-  <si>
-    <t>Product Backlog — 54 user stories (reference, edit Status / Owner / % freely)</t>
-  </si>
-  <si>
-    <t>Story</t>
-  </si>
-  <si>
-    <t>Pts</t>
-  </si>
-  <si>
-    <t>US-001</t>
-  </si>
-  <si>
-    <t>Functional Requirement Gathering</t>
-  </si>
-  <si>
-    <t>US-002</t>
-  </si>
-  <si>
-    <t>Business Requirement Analysis</t>
-  </si>
-  <si>
     <t>Requirement Clarification (A-8b)</t>
   </si>
   <si>
+    <t>Abe</t>
+  </si>
+  <si>
     <t>User Flow Definition</t>
   </si>
   <si>
@@ -425,6 +425,9 @@
     <t>HL Architecture</t>
   </si>
   <si>
+    <t>API Definition</t>
+  </si>
+  <si>
     <t>US-012</t>
   </si>
   <si>
@@ -782,25 +785,19 @@
     <t xml:space="preserve">  • Backlog         — reference list of all 54 user stories</t>
   </si>
   <si>
-    <t>Abe</t>
-  </si>
-  <si>
-    <t>Abe, Yash, Het</t>
-  </si>
-  <si>
-    <t>Het</t>
-  </si>
-  <si>
-    <t>Yash, Abe, Het</t>
-  </si>
-  <si>
-    <t>Yash, Abe</t>
-  </si>
-  <si>
-    <t>Abe, Yash</t>
-  </si>
-  <si>
-    <t>API Definition</t>
+    <t>Qdrant</t>
+  </si>
+  <si>
+    <t>Het will own UX design.</t>
+  </si>
+  <si>
+    <t>Yash, Het</t>
+  </si>
+  <si>
+    <t>DB schema</t>
+  </si>
+  <si>
+    <t>Built back-of-envelope cost model for both at 200 apps/hr.</t>
   </si>
 </sst>
 </file>
@@ -962,25 +959,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1094,6 +1091,13 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFF4A6A6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
@@ -1108,7 +1112,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF4A6A6"/>
+          <fgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1136,7 +1140,42 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4A6A6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1157,7 +1196,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
+          <fgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1165,48 +1204,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF4A6A6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1263,7 +1260,7 @@
   <c:date1904 val="0"/>
   <c:lang val="en-GB"/>
   <c:roundedCorners val="1"/>
-  <c:style val="11"/>
+  <c:style val="2"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -1343,7 +1340,7 @@
                   <c:v>0.48529411764705882</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.95</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1359,7 +1356,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-1DB4-7F4A-8888-4A2A4FDFBA65}"/>
+              <c16:uniqueId val="{00000000-2B40-E743-8325-8329E638FE01}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1794,146 +1791,146 @@
     <col min="7" max="8" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="24" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="17"/>
-      <c r="C7" s="19" t="s">
+      <c r="B7" s="16"/>
+      <c r="C7" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="17"/>
-      <c r="E7" s="19" t="s">
+      <c r="D7" s="16"/>
+      <c r="E7" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="17"/>
-      <c r="G7" s="19" t="s">
+      <c r="F7" s="16"/>
+      <c r="G7" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="17"/>
+      <c r="H7" s="16"/>
     </row>
     <row r="8" spans="1:8" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="17"/>
-      <c r="C8" s="16" t="str">
-        <f>ROUND('Sprint Tracker'!E3*100,0)&amp;"%"</f>
+      <c r="B8" s="16"/>
+      <c r="C8" s="15" t="str">
+        <f>ROUND('Sprint Tracker'!E4*100,0)&amp;"%"</f>
         <v>0%</v>
       </c>
-      <c r="D8" s="17"/>
-      <c r="E8" s="16">
+      <c r="D8" s="16"/>
+      <c r="E8" s="15">
         <f>COUNTA(Backlog!A4:A56)</f>
         <v>53</v>
       </c>
-      <c r="F8" s="17"/>
-      <c r="G8" s="16">
+      <c r="F8" s="16"/>
+      <c r="G8" s="15">
         <f>COUNTIF(Backlog!H4:H56,"Done")</f>
-        <v>2</v>
-      </c>
-      <c r="H8" s="17"/>
+        <v>14</v>
+      </c>
+      <c r="H8" s="16"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="19" t="s">
+      <c r="B10" s="16"/>
+      <c r="C10" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="17"/>
-      <c r="E10" s="19" t="s">
+      <c r="D10" s="16"/>
+      <c r="E10" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="17"/>
-      <c r="G10" s="19" t="s">
+      <c r="F10" s="16"/>
+      <c r="G10" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="H10" s="17"/>
+      <c r="H10" s="16"/>
     </row>
     <row r="11" spans="1:8" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="16">
+      <c r="A11" s="15">
         <f>COUNTIF(Blockers!G3:G48,"Open")+COUNTIF(Blockers!G3:G48,"In Progress")</f>
         <v>0</v>
       </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="16">
-        <f>COUNTIF('Pending Tasks'!H4:H98,"Not Started")+COUNTIF('Pending Tasks'!H4:H98,"In Progress")</f>
-        <v>6</v>
-      </c>
-      <c r="D11" s="17"/>
-      <c r="E11" s="16">
+      <c r="B11" s="16"/>
+      <c r="C11" s="15">
+        <f>COUNTIF('Pending Tasks'!H4:H96,"Not Started")+COUNTIF('Pending Tasks'!H4:H96,"In Progress")</f>
+        <v>4</v>
+      </c>
+      <c r="D11" s="16"/>
+      <c r="E11" s="15">
         <f>COUNTIF('High Priority'!E3:E48,"&lt;&gt;Closed")-COUNTBLANK('High Priority'!E3:E48)</f>
         <v>2</v>
       </c>
-      <c r="F11" s="17"/>
-      <c r="G11" s="16">
+      <c r="F11" s="16"/>
+      <c r="G11" s="15">
         <f ca="1">TODAY()-DATE(2026,6,22)</f>
-        <v>1</v>
-      </c>
-      <c r="H11" s="17"/>
+        <v>16</v>
+      </c>
+      <c r="H11" s="16"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-    </row>
-    <row r="15" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
+    </row>
+    <row r="15" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -1953,12 +1950,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B16" s="14" t="s">
         <v>20</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>21</v>
       </c>
       <c r="C16" s="4">
         <v>34</v>
@@ -1975,12 +1972,12 @@
         <v>In Progress</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C17" s="4">
         <v>39</v>
@@ -1989,17 +1986,16 @@
         <v>0</v>
       </c>
       <c r="E17" s="5">
-        <f>D17/C17</f>
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="F17" s="4" t="str">
         <f>IF(E17=1,"Done",IF(E17&gt;=0.7,"On Track",IF(E17&gt;=0.3,"In Progress",IF(E17&gt;0,"At Risk","Not Started"))))</f>
-        <v>Not Started</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>On Track</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>24</v>
@@ -2019,7 +2015,7 @@
         <v>Not Started</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>25</v>
       </c>
@@ -2041,7 +2037,7 @@
         <v>Not Started</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>27</v>
       </c>
@@ -2064,18 +2060,18 @@
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" s="12" t="s">
+      <c r="A40" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="B40" s="13"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="13"/>
-      <c r="F40" s="13"/>
-      <c r="G40" s="13"/>
-      <c r="H40" s="13"/>
-    </row>
-    <row r="41" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B40" s="14"/>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="14"/>
+      <c r="H40" s="14"/>
+    </row>
+    <row r="41" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>30</v>
       </c>
@@ -2101,23 +2097,23 @@
     <row r="42" spans="1:8" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="6">
         <f>IFERROR(INDEX('Daily Log'!A:A,MATCH(MAX('Daily Log'!A:A),'Daily Log'!A:A,0)),"—")</f>
-        <v>46195</v>
+        <v>46210</v>
       </c>
       <c r="B42" s="3" t="str">
         <f>IFERROR(INDEX('Daily Log'!B:B,MATCH(MAX('Daily Log'!A:A),'Daily Log'!A:A,0)),"—")</f>
-        <v>Sprint 0</v>
+        <v>Sprint 1</v>
       </c>
       <c r="C42" s="3" t="str">
         <f>IFERROR(INDEX('Daily Log'!C:C,MATCH(MAX('Daily Log'!A:A),'Daily Log'!A:A,0)),"—")</f>
-        <v>40%</v>
+        <v>100%</v>
       </c>
       <c r="D42" s="3" t="str">
         <f>IFERROR(INDEX('Daily Log'!D:D,MATCH(MAX('Daily Log'!A:A),'Daily Log'!A:A,0)),"—")</f>
-        <v>48%</v>
+        <v>100%</v>
       </c>
       <c r="E42" s="3" t="str">
         <f>IFERROR(INDEX('Daily Log'!E:E,MATCH(MAX('Daily Log'!A:A),'Daily Log'!A:A,0)),"—")</f>
-        <v>PRD v2.0 finalised; full Agile backlog authored (15 epics, 54 stories, 217 pts); Sprint 0–4 plan; repo initialised; A-8b drafted</v>
+        <v>Completed all remaining Sprint 1 stories (US-102-US-111): CSV ingestion + INCOMPLETE handling, placeholder risk scorer (A-8b compliant), 5-clause policy corpus, TF-IDF RAG retrieval (US-111 spike &gt;=85% accuracy), mock regulatory stub, recommendation engine with kill-switch, decision_record audit persistence, underwriter queue/detail/assess UI, demo script. Sprint 1 now 100% complete (39/39 pts, 11/11 stories).</v>
       </c>
       <c r="F42" s="3">
         <f>COUNTIF(Blockers!G:G,"Open")+COUNTIF(Blockers!G:G,"In Progress")</f>
@@ -2125,19 +2121,11 @@
       </c>
       <c r="G42" s="3" t="str">
         <f>IFERROR(INDEX('Daily Log'!H:H,MATCH(MAX('Daily Log'!A:A),'Daily Log'!A:A,0)),"—")</f>
-        <v>Yash, Abe, Het</v>
+        <v>Yash, Het</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="G10:H10"/>
     <mergeCell ref="A40:H40"/>
     <mergeCell ref="B16"/>
     <mergeCell ref="A3:H3"/>
@@ -2153,6 +2141,14 @@
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="G11:H11"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="G10:H10"/>
   </mergeCells>
   <conditionalFormatting sqref="F16:F20">
     <cfRule type="expression" dxfId="36" priority="1">
@@ -2178,7 +2174,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I199"/>
+  <dimension ref="A1:I200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2224,7 +2220,7 @@
         <v>46195</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>40</v>
@@ -2242,14 +2238,38 @@
         <v>43</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>250</v>
+        <v>44</v>
       </c>
       <c r="I2" s="8" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="9"/>
+    <row r="3" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+      <c r="A3" s="7">
+        <v>46210</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="4"/>
+      <c r="G3" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="9"/>
@@ -2818,26 +2838,37 @@
     <row r="192" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A192" s="9"/>
     </row>
-    <row r="193" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A193" s="9"/>
     </row>
-    <row r="194" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A194" s="9"/>
     </row>
-    <row r="195" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A195" s="9"/>
     </row>
-    <row r="196" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A196" s="9"/>
     </row>
-    <row r="197" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A197" s="9"/>
     </row>
-    <row r="198" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A198" s="9"/>
     </row>
-    <row r="199" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A199" s="9"/>
+    </row>
+    <row r="200" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A200" s="7"/>
+      <c r="B200" s="4"/>
+      <c r="C200" s="4"/>
+      <c r="D200" s="4"/>
+      <c r="E200" s="8"/>
+      <c r="F200" s="4"/>
+      <c r="G200" s="8"/>
+      <c r="H200" s="4"/>
+      <c r="I200" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2862,57 +2893,57 @@
   <sheetData>
     <row r="1" spans="1:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>35</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B2" s="7">
         <v>46195</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>56</v>
+        <v>251</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E2" s="22" t="s">
-        <v>248</v>
+        <v>59</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>60</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>57</v>
+        <v>252</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="I2" s="7"/>
     </row>
@@ -3298,31 +3329,31 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D198">
-    <cfRule type="expression" dxfId="31" priority="6">
-      <formula>$D2="Critical"</formula>
+    <cfRule type="expression" dxfId="31" priority="9">
+      <formula>$D2="Low"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="7">
+    <cfRule type="expression" dxfId="30" priority="8">
+      <formula>$D2="Medium"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="29" priority="7">
       <formula>$D2="High"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="8">
-      <formula>$D2="Medium"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="28" priority="9">
-      <formula>$D2="Low"</formula>
+    <cfRule type="expression" dxfId="28" priority="6">
+      <formula>$D2="Critical"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G198">
     <cfRule type="expression" dxfId="27" priority="1">
       <formula>$G2="Open"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="2">
-      <formula>$G2="In Progress"</formula>
+    <cfRule type="expression" dxfId="26" priority="4">
+      <formula>$G2="Closed"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="25" priority="3">
       <formula>$G2="Resolved"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="4">
-      <formula>$G2="Closed"</formula>
+    <cfRule type="expression" dxfId="24" priority="2">
+      <formula>$G2="In Progress"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="23" priority="5">
       <formula>$G2="Escalated"</formula>
@@ -3342,7 +3373,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:J197"/>
+  <dimension ref="A1:J195"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -3357,22 +3388,22 @@
   <sheetData>
     <row r="1" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>35</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>18</v>
@@ -3381,27 +3412,27 @@
         <v>19</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>249</v>
+        <v>71</v>
       </c>
       <c r="F2" s="7">
         <v>46196</v>
@@ -3410,30 +3441,30 @@
         <v>0.2</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="E3" s="4" t="s">
         <v>71</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>249</v>
       </c>
       <c r="F3" s="7">
         <v>46196</v>
@@ -3442,204 +3473,148 @@
         <v>0</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="J3" s="8"/>
     </row>
-    <row r="4" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>248</v>
+        <v>83</v>
       </c>
       <c r="F4" s="7">
         <v>46196</v>
       </c>
       <c r="G4" s="5">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B5" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>75</v>
-      </c>
       <c r="E5" s="4" t="s">
-        <v>251</v>
+        <v>49</v>
       </c>
       <c r="F5" s="7">
         <v>46196</v>
       </c>
       <c r="G5" s="5">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>252</v>
+        <v>60</v>
       </c>
       <c r="F6" s="7">
         <v>46196</v>
       </c>
       <c r="G6" s="5">
-        <v>0.1</v>
+        <v>0.9</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>44</v>
+        <v>78</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>60</v>
       </c>
       <c r="F7" s="7">
         <v>46196</v>
       </c>
       <c r="G7" s="5">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>248</v>
-      </c>
-      <c r="F8" s="7">
-        <v>46196</v>
-      </c>
-      <c r="G8" s="5">
-        <v>0.3</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B9" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E9" s="22" t="s">
-        <v>248</v>
-      </c>
-      <c r="F9" s="7">
-        <v>46196</v>
-      </c>
-      <c r="G9" s="5">
-        <v>0.6</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>93</v>
-      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F8" s="9"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F9" s="9"/>
+      <c r="G9" s="10"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F10" s="9"/>
@@ -4385,53 +4360,45 @@
       <c r="F195" s="9"/>
       <c r="G195" s="10"/>
     </row>
-    <row r="196" spans="6:7" x14ac:dyDescent="0.2">
-      <c r="F196" s="9"/>
-      <c r="G196" s="10"/>
-    </row>
-    <row r="197" spans="6:7" x14ac:dyDescent="0.2">
-      <c r="F197" s="9"/>
-      <c r="G197" s="10"/>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F298">
+  <conditionalFormatting sqref="F2:F296">
     <cfRule type="expression" dxfId="22" priority="8">
       <formula>AND($F2&lt;&gt;"",$F2&lt;TODAY(),$H2&lt;&gt;"Done")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H298">
-    <cfRule type="expression" dxfId="21" priority="1">
+  <conditionalFormatting sqref="H2:H296">
+    <cfRule type="expression" dxfId="21" priority="2">
+      <formula>$H2="In Progress"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="20" priority="3">
+      <formula>$H2="Blocked"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="19" priority="4">
+      <formula>$H2="Not Started"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="18" priority="1">
       <formula>$H2="Done"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="2">
-      <formula>$H2="In Progress"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="19" priority="3">
-      <formula>$H2="Blocked"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="18" priority="4">
-      <formula>$H2="Not Started"</formula>
-    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I298">
-    <cfRule type="expression" dxfId="17" priority="5">
-      <formula>$I2="High"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="16" priority="6">
+  <conditionalFormatting sqref="I2:I296">
+    <cfRule type="expression" dxfId="17" priority="6">
       <formula>$I2="Medium"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="7">
+    <cfRule type="expression" dxfId="16" priority="7">
       <formula>$I2="Low"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="5">
+      <formula>$I2="High"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="H2:H298" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="H2:H296" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"Not Started,In Progress,Blocked,Done,Cancelled"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I2:I298" xr:uid="{00000000-0002-0000-0300-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I2:I296" xr:uid="{00000000-0002-0000-0300-000001000000}">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C2:C298" xr:uid="{00000000-0002-0000-0300-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="C2:C296" xr:uid="{00000000-0002-0000-0300-000002000000}">
       <formula1>"Sprint 0,Sprint 1,Sprint 2,Sprint 3,Sprint 4"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4455,94 +4422,94 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>35</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D2" s="7">
         <v>46196</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>101</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>102</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>104</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>105</v>
       </c>
       <c r="D3" s="7">
         <v>46196</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>107</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>108</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>110</v>
       </c>
       <c r="D4" s="7">
         <v>46197</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -4892,27 +4859,27 @@
         <v>18</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" s="4">
         <v>34</v>
@@ -4941,28 +4908,27 @@
         <v>In Progress</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C3" s="4">
         <v>39</v>
       </c>
       <c r="D3" s="4">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="E3" s="5">
-        <f>D3/C3</f>
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="F3" s="4">
         <v>11</v>
       </c>
       <c r="G3" s="4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H3" s="7">
         <v>46202</v>
@@ -4972,12 +4938,12 @@
       </c>
       <c r="J3" s="4" t="str">
         <f>IF(E3=1,"Done",IF(E3&gt;=0.7,"On Track",IF(E3&gt;=0.3,"In Progress",IF(E3&gt;0,"At Risk","Not Started"))))</f>
-        <v>Not Started</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>On Track</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>24</v>
@@ -5009,7 +4975,7 @@
         <v>Not Started</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>25</v>
       </c>
@@ -5043,7 +5009,7 @@
         <v>Not Started</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>27</v>
       </c>
@@ -5114,37 +5080,37 @@
     <col min="9" max="9" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="21" t="s">
-        <v>117</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
+    <row r="1" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D2" t="s">
         <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G2" t="s">
         <v>35</v>
@@ -5158,22 +5124,22 @@
     </row>
     <row r="3" spans="1:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>14</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>35</v>
@@ -5185,268 +5151,268 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E4" s="4">
         <v>3</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G4" s="22" t="s">
-        <v>248</v>
+        <v>59</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>60</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I4" s="5">
         <v>0.75</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E5" s="4">
         <v>3</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G5" s="22" t="s">
-        <v>248</v>
+        <v>59</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>60</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I5" s="5">
         <v>0.7</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>89</v>
-      </c>
       <c r="C6" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E6" s="4">
         <v>3</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>248</v>
+        <v>60</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I6" s="5">
         <v>0.3</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>92</v>
-      </c>
       <c r="C7" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E7" s="4">
         <v>2</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G7" s="22" t="s">
-        <v>248</v>
+        <v>59</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>60</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I7" s="5">
         <v>0.6</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>87</v>
+        <v>122</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E8" s="4">
         <v>2</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G8" s="22" t="s">
-        <v>247</v>
+        <v>59</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>124</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I8" s="5">
         <v>0.4</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>125</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E9" s="4">
         <v>3</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>249</v>
+        <v>71</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I9" s="5">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>68</v>
-      </c>
       <c r="D10" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E10" s="4">
         <v>3</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>249</v>
+        <v>71</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I10" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>126</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E11" s="4">
         <v>3</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>248</v>
+        <v>60</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I11" s="5">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>127</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E12" s="4">
         <v>3</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>251</v>
+        <v>60</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>58</v>
+        <v>133</v>
       </c>
       <c r="I12" s="5">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>80</v>
       </c>
@@ -5457,689 +5423,711 @@
         <v>82</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E13" s="4">
         <v>3</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>248</v>
+        <v>60</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I13" s="5">
         <v>0.1</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>84</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>253</v>
+        <v>128</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E14" s="4">
         <v>3</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>252</v>
+        <v>83</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I14" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E15" s="4">
         <v>2</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>248</v>
+        <v>60</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I15" s="5">
         <v>0.85</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E16" s="4">
         <v>3</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I16" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E17" s="4">
         <v>2</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I17" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E18" s="4">
         <v>3</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G18" s="4"/>
+        <v>59</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>49</v>
+      </c>
       <c r="H18" s="4" t="s">
-        <v>72</v>
+        <v>133</v>
       </c>
       <c r="I18" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E19" s="4">
         <v>3</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G19" s="4"/>
+        <v>59</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>124</v>
+      </c>
       <c r="H19" s="4" t="s">
-        <v>72</v>
+        <v>133</v>
       </c>
       <c r="I19" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E20" s="4">
         <v>5</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G20" s="4"/>
+        <v>59</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>71</v>
+      </c>
       <c r="H20" s="4" t="s">
-        <v>72</v>
+        <v>133</v>
       </c>
       <c r="I20" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E21" s="4">
         <v>2</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G21" s="4"/>
+        <v>59</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>49</v>
+      </c>
       <c r="H21" s="4" t="s">
-        <v>72</v>
+        <v>133</v>
       </c>
       <c r="I21" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="B22" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>146</v>
-      </c>
       <c r="D22" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E22" s="4">
         <v>5</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G22" s="4"/>
+        <v>59</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="H22" s="4" t="s">
-        <v>72</v>
+        <v>133</v>
       </c>
       <c r="I22" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E23" s="4">
         <v>5</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G23" s="4"/>
+        <v>59</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>60</v>
+      </c>
       <c r="H23" s="4" t="s">
-        <v>72</v>
+        <v>133</v>
       </c>
       <c r="I23" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E24" s="4">
         <v>5</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G24" s="4"/>
+        <v>59</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>71</v>
+      </c>
       <c r="H24" s="4" t="s">
-        <v>72</v>
+        <v>133</v>
       </c>
       <c r="I24" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>82</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E25" s="4">
         <v>3</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G25" s="4"/>
+        <v>59</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>49</v>
+      </c>
       <c r="H25" s="4" t="s">
-        <v>72</v>
+        <v>133</v>
       </c>
       <c r="I25" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E26" s="4">
         <v>3</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="G26" s="4"/>
+        <v>76</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>49</v>
+      </c>
       <c r="H26" s="4" t="s">
-        <v>72</v>
+        <v>133</v>
       </c>
       <c r="I26" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E27" s="4">
         <v>2</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G27" s="4"/>
+        <v>59</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>60</v>
+      </c>
       <c r="H27" s="4" t="s">
-        <v>72</v>
+        <v>133</v>
       </c>
       <c r="I27" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E28" s="4">
         <v>3</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G28" s="4"/>
+        <v>59</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>60</v>
+      </c>
       <c r="H28" s="4" t="s">
-        <v>72</v>
+        <v>133</v>
       </c>
       <c r="I28" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="E29" s="4">
         <v>8</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I29" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="E30" s="4">
         <v>5</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I30" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="E31" s="4">
         <v>5</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G31" s="4"/>
       <c r="H31" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I31" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="E32" s="4">
         <v>5</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G32" s="4"/>
       <c r="H32" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I32" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="E33" s="4">
         <v>5</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I33" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="E34" s="4">
         <v>8</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I34" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="E35" s="4">
         <v>3</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I35" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="E36" s="4">
         <v>5</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I36" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="E37" s="4">
         <v>3</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I37" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>25</v>
@@ -6148,25 +6136,25 @@
         <v>3</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I38" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="C39" s="4" t="s">
         <v>187</v>
-      </c>
-      <c r="B39" s="8" t="s">
-        <v>188</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>186</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>25</v>
@@ -6175,25 +6163,25 @@
         <v>8</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G39" s="4"/>
       <c r="H39" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I39" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>25</v>
@@ -6202,25 +6190,25 @@
         <v>8</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G40" s="4"/>
       <c r="H40" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I40" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>25</v>
@@ -6229,25 +6217,25 @@
         <v>8</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G41" s="4"/>
       <c r="H41" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I41" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="C42" s="4" t="s">
         <v>194</v>
-      </c>
-      <c r="B42" s="8" t="s">
-        <v>195</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>193</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>25</v>
@@ -6256,25 +6244,25 @@
         <v>3</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="G42" s="4"/>
       <c r="H42" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I42" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D43" s="4" t="s">
         <v>25</v>
@@ -6283,25 +6271,25 @@
         <v>5</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I43" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D44" s="4" t="s">
         <v>25</v>
@@ -6310,25 +6298,25 @@
         <v>5</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G44" s="4"/>
       <c r="H44" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I44" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D45" s="4" t="s">
         <v>25</v>
@@ -6337,25 +6325,25 @@
         <v>3</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G45" s="4"/>
       <c r="H45" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I45" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>25</v>
@@ -6364,22 +6352,22 @@
         <v>5</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G46" s="4"/>
       <c r="H46" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I46" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>82</v>
@@ -6391,25 +6379,25 @@
         <v>8</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G47" s="4"/>
       <c r="H47" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I47" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>27</v>
@@ -6418,25 +6406,25 @@
         <v>5</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G48" s="4"/>
       <c r="H48" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I48" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>27</v>
@@ -6445,25 +6433,25 @@
         <v>5</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G49" s="4"/>
       <c r="H49" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I49" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>27</v>
@@ -6472,25 +6460,25 @@
         <v>5</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G50" s="4"/>
       <c r="H50" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I50" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>27</v>
@@ -6499,25 +6487,25 @@
         <v>5</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G51" s="4"/>
       <c r="H51" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I51" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>27</v>
@@ -6526,25 +6514,25 @@
         <v>3</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G52" s="4"/>
       <c r="H52" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I52" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D53" s="4" t="s">
         <v>27</v>
@@ -6553,25 +6541,25 @@
         <v>5</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G53" s="4"/>
       <c r="H53" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I53" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>27</v>
@@ -6580,25 +6568,25 @@
         <v>8</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G54" s="4"/>
       <c r="H54" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I54" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D55" s="4" t="s">
         <v>27</v>
@@ -6607,25 +6595,25 @@
         <v>3</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G55" s="4"/>
       <c r="H55" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I55" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>27</v>
@@ -6634,11 +6622,11 @@
         <v>3</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="G56" s="4"/>
       <c r="H56" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I56" s="5">
         <v>0</v>
@@ -7108,134 +7096,134 @@
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="24" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
-        <v>225</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
+    <row r="1" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="11"/>
     </row>
-    <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="11"/>
     </row>
-    <row r="10" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="11"/>
     </row>
-    <row r="12" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="11"/>
     </row>
-    <row r="18" spans="1:1" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="11"/>
     </row>
-    <row r="20" spans="1:1" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" ht="16" x14ac:dyDescent="0.2">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" ht="16" x14ac:dyDescent="0.2">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" ht="16" x14ac:dyDescent="0.2">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" ht="16" x14ac:dyDescent="0.2">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" ht="16" x14ac:dyDescent="0.2">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" ht="16" x14ac:dyDescent="0.2">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="11" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" ht="16" x14ac:dyDescent="0.2">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="11" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>

</xml_diff>